<commit_message>
Add Towns tab to data.xlsx
Headers: Town ID (A1), Town Name (B1).

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data.xlsx
+++ b/data.xlsx
@@ -8,6 +8,7 @@
   </bookViews>
   <sheets>
     <sheet name="Sheet" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Towns" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -418,4 +419,30 @@
   <sheetData/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:B1"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>Town ID</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>Town Name</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
Populate Locations sheet with original Kanto-inspired location names
Add 51 towns, trails, and destinations with original names, types,
and IDs replacing the Pokemon Red/Blue location references.

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data.xlsx
+++ b/data.xlsx
@@ -8,7 +8,7 @@
   </bookViews>
   <sheets>
     <sheet name="Sheet" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="Towns" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="Locations" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -427,18 +427,788 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B1"/>
+  <dimension ref="A1:C52"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="inlineStr">
         <is>
-          <t>Town ID</t>
+          <t>Location ID</t>
         </is>
       </c>
       <c r="B1" t="inlineStr">
         <is>
-          <t>Town Name</t>
+          <t>Location Name</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>Location Type</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="n">
+        <v>1</v>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>Meadowbrook</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>Town</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="n">
+        <v>2</v>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>Sproutwood Trail</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>Trail</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="n">
+        <v>3</v>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>Maple City</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>Town</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="n">
+        <v>4</v>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>Timberline Trail</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>Trail</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="n">
+        <v>5</v>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>Thornwood Forest</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>Destination</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="n">
+        <v>6</v>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>Ironvale</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>Town</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="n">
+        <v>7</v>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>Cragpass Trail</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>Trail</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="n">
+        <v>8</v>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>Lunarpeak Cavern</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>Destination</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="n">
+        <v>9</v>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>Moonshadow Trail</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>Trail</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="n">
+        <v>10</v>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>Azuremere City</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>Town</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="n">
+        <v>11</v>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>Brightwater Bridge</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>Trail</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="n">
+        <v>12</v>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>Tidecrest Trail</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>Trail</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="n">
+        <v>13</v>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>Fernway Trail</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>Trail</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="n">
+        <v>14</v>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>Hollowpass Tunnel</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>Trail</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="n">
+        <v>15</v>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>Sunreach Trail</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>Trail</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="n">
+        <v>16</v>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>Scarletide City</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>Town</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="n">
+        <v>17</v>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>The Gilded Voyager</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>Destination</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="n">
+        <v>18</v>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>Portside Trail</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>Trail</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="n">
+        <v>19</v>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>Molehill Depths</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>Destination</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="n">
+        <v>20</v>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>Stonewind Trail</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>Trail</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="n">
+        <v>21</v>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>Cindercross Trail</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>Trail</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="n">
+        <v>22</v>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>Shadowrock Tunnel</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>Destination</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="n">
+        <v>23</v>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>Voltspire Station</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>Destination</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="n">
+        <v>24</v>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>Ashen Trail</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>Trail</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="n">
+        <v>25</v>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>Duskpass Tunnel</t>
+        </is>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>Trail</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="n">
+        <v>26</v>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>Willowshade Trail</t>
+        </is>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>Trail</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="n">
+        <v>27</v>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>Jadespire City</t>
+        </is>
+      </c>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>Town</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="n">
+        <v>28</v>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>Greenridge Trail</t>
+        </is>
+      </c>
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>Trail</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="n">
+        <v>29</v>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>The Red Line</t>
+        </is>
+      </c>
+      <c r="C30" t="inlineStr">
+        <is>
+          <t>Trail</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="n">
+        <v>30</v>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>Windrush Trail</t>
+        </is>
+      </c>
+      <c r="C31" t="inlineStr">
+        <is>
+          <t>Trail</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="n">
+        <v>31</v>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>Rosemire City</t>
+        </is>
+      </c>
+      <c r="C32" t="inlineStr">
+        <is>
+          <t>Town</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="n">
+        <v>32</v>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>Wildmere Reserve</t>
+        </is>
+      </c>
+      <c r="C33" t="inlineStr">
+        <is>
+          <t>Destination</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="n">
+        <v>33</v>
+      </c>
+      <c r="B34" t="inlineStr">
+        <is>
+          <t>Marshlight Trail</t>
+        </is>
+      </c>
+      <c r="C34" t="inlineStr">
+        <is>
+          <t>Trail</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="n">
+        <v>34</v>
+      </c>
+      <c r="B35" t="inlineStr">
+        <is>
+          <t>Reedhollow Trail</t>
+        </is>
+      </c>
+      <c r="C35" t="inlineStr">
+        <is>
+          <t>Trail</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="n">
+        <v>35</v>
+      </c>
+      <c r="B36" t="inlineStr">
+        <is>
+          <t>Driftgrass Trail</t>
+        </is>
+      </c>
+      <c r="C36" t="inlineStr">
+        <is>
+          <t>Trail</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="n">
+        <v>36</v>
+      </c>
+      <c r="B37" t="inlineStr">
+        <is>
+          <t>Slumberreed Trail</t>
+        </is>
+      </c>
+      <c r="C37" t="inlineStr">
+        <is>
+          <t>Trail</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="n">
+        <v>37</v>
+      </c>
+      <c r="B38" t="inlineStr">
+        <is>
+          <t>Duskthistle Town</t>
+        </is>
+      </c>
+      <c r="C38" t="inlineStr">
+        <is>
+          <t>Town</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="n">
+        <v>38</v>
+      </c>
+      <c r="B39" t="inlineStr">
+        <is>
+          <t>Spire of Echoes</t>
+        </is>
+      </c>
+      <c r="C39" t="inlineStr">
+        <is>
+          <t>Destination</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="n">
+        <v>39</v>
+      </c>
+      <c r="B40" t="inlineStr">
+        <is>
+          <t>Amberspire City</t>
+        </is>
+      </c>
+      <c r="C40" t="inlineStr">
+        <is>
+          <t>Town</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="n">
+        <v>40</v>
+      </c>
+      <c r="B41" t="inlineStr">
+        <is>
+          <t>Helion Tower</t>
+        </is>
+      </c>
+      <c r="C41" t="inlineStr">
+        <is>
+          <t>Destination</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="n">
+        <v>41</v>
+      </c>
+      <c r="B42" t="inlineStr">
+        <is>
+          <t>Coralbreeze Trail</t>
+        </is>
+      </c>
+      <c r="C42" t="inlineStr">
+        <is>
+          <t>Trail</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="n">
+        <v>42</v>
+      </c>
+      <c r="B43" t="inlineStr">
+        <is>
+          <t>Saltspray Trail</t>
+        </is>
+      </c>
+      <c r="C43" t="inlineStr">
+        <is>
+          <t>Trail</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="n">
+        <v>43</v>
+      </c>
+      <c r="B44" t="inlineStr">
+        <is>
+          <t>Frostcoral Isles</t>
+        </is>
+      </c>
+      <c r="C44" t="inlineStr">
+        <is>
+          <t>Destination</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="n">
+        <v>44</v>
+      </c>
+      <c r="B45" t="inlineStr">
+        <is>
+          <t>Ember Town</t>
+        </is>
+      </c>
+      <c r="C45" t="inlineStr">
+        <is>
+          <t>Town</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="n">
+        <v>45</v>
+      </c>
+      <c r="B46" t="inlineStr">
+        <is>
+          <t>The Cinderkeep Manor</t>
+        </is>
+      </c>
+      <c r="C46" t="inlineStr">
+        <is>
+          <t>Destination</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="n">
+        <v>46</v>
+      </c>
+      <c r="B47" t="inlineStr">
+        <is>
+          <t>Driftwave Trail</t>
+        </is>
+      </c>
+      <c r="C47" t="inlineStr">
+        <is>
+          <t>Trail</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" t="n">
+        <v>47</v>
+      </c>
+      <c r="B48" t="inlineStr">
+        <is>
+          <t>Bramblecrest Trail</t>
+        </is>
+      </c>
+      <c r="C48" t="inlineStr">
+        <is>
+          <t>Trail</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" t="n">
+        <v>48</v>
+      </c>
+      <c r="B49" t="inlineStr">
+        <is>
+          <t>Stonegate Trail</t>
+        </is>
+      </c>
+      <c r="C49" t="inlineStr">
+        <is>
+          <t>Trail</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" t="n">
+        <v>49</v>
+      </c>
+      <c r="B50" t="inlineStr">
+        <is>
+          <t>Ascension Pass</t>
+        </is>
+      </c>
+      <c r="C50" t="inlineStr">
+        <is>
+          <t>Trail</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" t="n">
+        <v>50</v>
+      </c>
+      <c r="B51" t="inlineStr">
+        <is>
+          <t>The Summit</t>
+        </is>
+      </c>
+      <c r="C51" t="inlineStr">
+        <is>
+          <t>Destination</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" t="n">
+        <v>51</v>
+      </c>
+      <c r="B52" t="inlineStr">
+        <is>
+          <t>Champion's Cave</t>
+        </is>
+      </c>
+      <c r="C52" t="inlineStr">
+        <is>
+          <t>Destination</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Rename three locations in data.xlsx
Cragpass Trail -> Ashland Trail
Lunarpeak Cavern -> Lake Ashland Cavern
Azuremere City -> Sendai City

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data.xlsx
+++ b/data.xlsx
@@ -543,7 +543,7 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>Cragpass Trail</t>
+          <t>Ashland Trail</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
@@ -558,7 +558,7 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Lunarpeak Cavern</t>
+          <t>Lake Ashland Cavern</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
@@ -588,7 +588,7 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>Azuremere City</t>
+          <t>Sendai City</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">

</xml_diff>

<commit_message>
Restore the Quests tab in data.xlsx
The Quests tab (Questline_ID ... Text headers) was missing from the working
copy of data.xlsx and was left out of the previous commit; restored from the
earlier committed version, in its original spot before Openings.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data.xlsx
+++ b/data.xlsx
@@ -5,7 +5,8 @@
   <sheets>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Locations" sheetId="1" state="visible" r:id="rId1"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Location_1" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Openings" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Quests" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Openings" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -8742,6 +8743,66 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
+  <dimension ref="A1:H1"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="13.38" customWidth="1" style="5" min="2" max="2"/>
+    <col width="13.88" customWidth="1" style="5" min="3" max="3"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Questline_ID</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>Questline_Name</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>Sequence_Name</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>Location(s)</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>Modifiers</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>Triggered</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>Action</t>
+        </is>
+      </c>
+      <c r="H1" s="1" t="inlineStr">
+        <is>
+          <t>Text</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
   <dimension ref="A1:Z220"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="12.63" defaultRowHeight="15" customHeight="1"/>
   <cols>
@@ -8837,7 +8898,7 @@
       <c r="Z2" s="2" t="n"/>
     </row>
     <row r="3" ht="12.75" customHeight="1" s="5">
-      <c r="A3" t="n">
+      <c r="A3" s="0" t="n">
         <v>2</v>
       </c>
       <c r="B3" s="2" t="inlineStr">

</xml_diff>